<commit_message>
Update multi-country benchmark workbook
</commit_message>
<xml_diff>
--- a/SurveyData_MultiCountry.xlsx
+++ b/SurveyData_MultiCountry.xlsx
@@ -2,19 +2,19 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read Me" sheetId="1" r:id="Rcf51c3f3bf704c8e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Item Crosswalk" sheetId="2" r:id="Rb69f7a2aef2e4512"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Q1 Internet Use" sheetId="3" r:id="Rdae75087b57143c0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Q10d Software Skills" sheetId="4" r:id="Rb4df1eff27454043"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Q17a Tech Easier" sheetId="5" r:id="Ra90c68aca8364c13"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Q20 Political News" sheetId="6" r:id="Rd6aadafd609b43df"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Q23a Petition" sheetId="7" r:id="R7281804272bb45f1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Q28a Surveillance" sheetId="8" r:id="Rb9699b59bcc147fa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Q34 Digital Benefits" sheetId="9" r:id="R8d884d285b70454f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Q36a Medical Robot" sheetId="10" r:id="R351d75d51c084a83"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Distributions Long" sheetId="11" r:id="R942751c8e1644855"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Q10d Routing" sheetId="12" r:id="Rb41b733f9443406b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Language Weights QA" sheetId="13" r:id="R74bb3818715e410c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read Me" sheetId="1" r:id="Rf72335bcf0a84fba"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Item Crosswalk" sheetId="2" r:id="Rdc0f587ddd654d40"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Q1 Internet Use" sheetId="3" r:id="Rcbc4ef89f131450a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Q10d Software Skills" sheetId="4" r:id="R5284febfb6e04861"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Q17a Tech Easier" sheetId="5" r:id="Redb1448c5d714004"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Q20 Political News" sheetId="6" r:id="R5e5ffdd547314c83"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Q23a Petition" sheetId="7" r:id="R8c2fd72904904250"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Q28a Surveillance" sheetId="8" r:id="Rdba050e5e1b046ac"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Q34 Digital Benefits" sheetId="9" r:id="R876b170cf9894254"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Q36a Medical Robot" sheetId="10" r:id="R298b51fdbf6d4a8c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Distributions Long" sheetId="11" r:id="R66091354b9564b1d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Q10d Routing" sheetId="12" r:id="R0b728610b3d140d3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Language Weights QA" sheetId="13" r:id="R1366a9f951954fb0"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -722,7 +722,7 @@
         <x:v>Language composition</x:v>
       </x:c>
       <x:c r="B6" s="6" t="str">
-        <x:v>Switzerland full sample: German 2,129; French 731; Italian 168. USA full sample: English 1,534; Spanish 56. Canada is restricted to the observed INTLANG value eng (English), N=1,342; literal eng matches zero records.</x:v>
+        <x:v>Switzerland full sample: German 2,129; French 731; Italian 168; N=3,028. HISTORICAL full multilingual sample; not the current language-matched benchmark. Current benchmark: INTLANG == deu (German), N=2,129, in SurveyData_MultiCountry_LanguageMatched.xlsx. USA full sample: English 1,534; Spanish 56. Canada is restricted to the observed INTLANG value eng (English), N=1,342; literal eng matches zero records.</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="38" customHeight="1">
@@ -4729,7 +4729,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3398ac19969a4fb9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R958756bc686d44b3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -27011,7 +27011,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R21bb565d75ee4ab0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R63d22e3292c04c03"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -49789,8 +49789,8 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="2">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R52066900133544b5"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R162b436cb48940ae"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rce116defee5f4532"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3d82343c66374721"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -52385,10 +52385,10 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="4">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9cc99bc07f2a4d96"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2b4ee79effe34be4"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8e0a7d76296149de"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf22986d1bb6548f4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R267f1412609b47b8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R803ff11d17c640fa"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfcea3f17bca54563"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R88762169fed84939"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -54720,7 +54720,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8980c2b7ef0f417d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7afed04216da4253"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -57176,7 +57176,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4fc56034ecd944b4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R71b62c1297ee4437"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -59584,7 +59584,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R77043d4c1af84374"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R338dc8d2d4ec453c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -61716,7 +61716,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc7653ee5c9394cb7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R836c9b7b26e24a5f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -64424,7 +64424,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc78d441214834620"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb2176a79c1344fae"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -66256,7 +66256,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9e912e6906c64e43"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbd1c7e2321594d9d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -68088,7 +68088,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd2ed87eec76d41ad"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc0990fcab7324940"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -69920,7 +69920,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R25f62fe3fc944f4a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2f378e6b801e4efa"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>